<commit_message>
Update the change register and conformance table for the release candidate.
CR-012 now includes administrators, CR-013 drops FR-009 and FR-013, and the new CR-015 records the ADR-006 differences (POST, GUID ids).
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-Change-Register-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-Change-Register-v3.0.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Target stays 3 s at 1,000 requests. Seeding method: app/db/seed/seed_requests.sql (1,000 rows, development or test database only). Verified by PT-01, not yet run (B2).</t>
+          <t>Target stays 3 s at 1,000 requests. PT-01 seeds 1,000 requests through the API (Test/Performance/PT-01_queue.sh) and passed: p95 0.064 s with 5 users (Test/Evidence/PT-01_Results.md). Measured locally; staging pending (B2).</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Reword AC-014.2: "Given a staff member who does not own the request, or whose category scope does not cover it, when they attempt to close, then the action is blocked (RBAC)." There is no separate close permission.</t>
+          <t>Reword AC-014.2: "Given a staff member who does not own the request or whose category scope does not cover it, and who is not an administrator, when they attempt to close, then the action is blocked (RBAC)." There is no separate close permission.</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Implemented rule: only the owning, in-scope staff member may close (RequestAccess.MayWorkOn); UT-04 8/8 passed. Closes scope freeze B4.</t>
+          <t>Built rule: the owning, in-scope staff member or an administrator may close (AuthorisationPolicy). IT-03 and AuthorisationTests pass; administrator close passes in acceptance. Closes scope freeze B4.</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Proposed for the scope freeze meeting, 2026-10-13, M. Malope</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>FR-009, FR-013, FR-015, FR-016, FR-017, FR-019, FR-020, FR-021</t>
+          <t>FR-015, FR-016, FR-017, FR-019, FR-020, FR-021</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Not built in app/ by the freeze (Scope Freeze v1.0). They carry no M3 verification claim.</t>
+          <t>Not built by the freeze (Scope Freeze v2.0). FR-009 and FR-013 were built after the freeze and left this CR. The rest carry no M3 verification claim.</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Proposed for the scope freeze meeting, 2026-10-13, M. Malope</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Record that the M3 RC is one deployable: the Razor Pages read the database directly (Staff/Queue, Staff/Details), not through a separate frontend deployable and the Requests service API.</t>
+          <t>Record that the M3 release candidate runs as one deployable: the web pages and the API share one application, not a separate frontend calling the Requests service. The pages already go through Application services and the queue repository.</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1176,12 +1176,54 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Found while building FR-008 (2026-10-12). Requirements are unaffected; the deviation is architectural.</t>
+          <t>Found while building FR-008 and rechecked after the merge with main. Requirements are unaffected; the deviation is architectural.</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Raised for K. Marota to decide, 2026-10-12, M. Malope</t>
+          <t>Raised for K. Marota to decide, 2026-10-13, M. Malope</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CR-015</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>ADR-006; Docs/API/openapi.yaml; FR-012; FR-002</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Align the ADR-006 contract with the built API: status changes use POST /api/v1/requests/{id}/status (the contract says PATCH), and category ids are GUIDs (the contract says integers).</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>K. Marota</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Decide: update ADR-006 and openapi.yaml, or change the API</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>The team accepted the POST route with the merged backend work; the GUID ids come from the data model. The API tests (IT-01, IT-03, ApiTests) use the built contract.</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Raised for K. Marota to decide, 2026-10-13, M. Malope</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the RTM and change register for the release candidate
Marks the requirements built after the scope freeze as in scope through the new CR-016, each traced to the tests that verify it (211/211 pass). CR-013 is withdrawn as superseded, and CR-005, CR-006, CR-007 and CR-009 are recorded as approved and implemented.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-Change-Register-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-Change-Register-v3.0.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -588,7 +588,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>PED v3 NFR-002 already reads 15 s. NFR-002 is out of M3 scope (Scope Freeze v1.0), so it is not verified in M3.</t>
+          <t>PED v3 NFR-002 reads 15 s. NFR-002 is now built (5 s polling) and verified by UpdatesPollingTests (CR-016).</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>M3 runs on the development identity, which Program.cs allows only in Development. Residual risk RSK-012. Blocks staging (B2) until closed.</t>
+          <t>M3 runs on the development identity, which Program.cs allows only in Development. Residual risk RSK-012. Blocks staging (B2) until closed. AC-019.1 and AC-020.1 are verified against the development sign-in only.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Deferred to M4</t>
+          <t>Approved and implemented: each category has a target response time in hours (default 72, set by administrators); a request's due time is fixed when it is submitted</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>FR-016 is out of M3 scope (CR-013).</t>
+          <t>Built in the release candidate (TargetResponseAtUtc, migration AddRemainingRequirements). Evidence: ResponseTargetTests, CategoryServiceTests, ReportingTests (AC-016.2) pass, 16 Oct 2026.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Decided 2026-10-14, M. Malope; for team sign-off with CR-016</t>
         </is>
       </c>
     </row>
@@ -793,17 +793,17 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Deferred to M4</t>
+          <t>Approved and implemented: CSV export of the performance table and of the matching requests, with the same filters as the page</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>FR-018 is out of M3 scope (Scope Freeze v1.0).</t>
+          <t>The export matches the display row for row (ReportingTests, AC-018.2), 16 Oct 2026.</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Decided 2026-10-14, M. Malope; for team sign-off with CR-016</t>
         </is>
       </c>
     </row>
@@ -835,17 +835,17 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Deferred to M4</t>
+          <t>Approved and implemented: a Sponsor role with its own summary page that reuses the management figures at summary level</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>FR-023 is out of M3 scope (Scope Freeze v1.0).</t>
+          <t>Pages/Reports/Summary; sponsors see no request details (ReportingTests AC-023.1, RequestAccessTests), 16 Oct 2026. Adds a fifth role, Sponsor, to the roles in ADR-005.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Decided 2026-10-14, M. Malope; for team sign-off with CR-016</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Initial list: Fault, Equipment, Security, IT, Maintenance, Lost Property, Other (AC-002.1). Held as reference data (Category) and seeded (DevelopmentSeed). Maintenance (FR-021) is deferred (CR-013).</t>
+          <t>Initial list: Fault, Equipment, Security, IT, Maintenance, Lost Property, Other (AC-002.1). Held as reference data (Category) and seeded (DevelopmentSeed). Maintenance by administrators (FR-021) is built (CR-016).</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -919,17 +919,17 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Deferred to M4</t>
+          <t>Approved and implemented: Rejected is terminal, reachable only from Received, and always carries a reason the requester sees</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>The app/ lifecycle has no Rejected status (RequestStatus, StatusTransition); it exists only in Backend/. AC-007.2 cannot be verified in M3.</t>
+          <t>RequestStatus.Rejected, StatusTransition, StatusTransitionService.RejectAsync; database check constraints widened (migration AddRemainingRequirements). Evidence: StatusTransitionTests, StatusTransitionServiceTests (AC-007.2), UpdatesPollingTests pass, 16 Oct 2026.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-12, M. Malope</t>
+          <t>Decided 2026-10-14, M. Malope; for team sign-off with CR-016</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1129,17 +1129,17 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Approve</t>
+          <t>Withdrawn: superseded by CR-016</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Not built by the freeze (Scope Freeze v2.0). FR-009 and FR-013 were built after the freeze and left this CR. The rest carry no M3 verification claim.</t>
+          <t>Every requirement it deferred (FR-015, FR-016, FR-017, FR-019, FR-020, FR-021) was built and verified before the release candidate, so nothing is deferred to M4.</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Proposed for the scope freeze meeting, 2026-10-13, M. Malope</t>
+          <t>Withdrawn 2026-10-16, M. Malope</t>
         </is>
       </c>
     </row>
@@ -1224,6 +1224,48 @@
       <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Raised for K. Marota to decide, 2026-10-13, M. Malope</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>CR-016</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>FR-005, FR-006, FR-015 to FR-023, NFR-002, NFR-007, NFR-008; supersedes CR-013; Scope Freeze v2.0</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Bring the work built after the scope freeze into the M3 release candidate, so the release candidate's scope is what was built and verified. Priorities and acceptance criteria are unchanged.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>All these requirements are built with automated tests: 211/211 pass locally on 16 Oct 2026 (RTM v3.0 shows each test). Limits: real sign-in is CR-003, so AC-019.1 and AC-020.1 are verified against the development sign-in only; nothing is deployed yet (B2).</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Proposed for team sign-off, 2026-10-16, M. Malope</t>
         </is>
       </c>
     </row>

</xml_diff>